<commit_message>
add ex1 more tries
</commit_message>
<xml_diff>
--- a/ex_res_1_after_fix.xlsx
+++ b/ex_res_1_after_fix.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\DataStructuresHW\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F47CF7A-B387-440F-80CE-569E22EBE573}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEDA6BD4-8A97-4A7F-A92C-01D426D3794A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="5844" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -383,10 +383,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="5" max="5" width="15" customWidth="1"/>
+    <col min="6" max="6" width="13.5" customWidth="1"/>
     <col min="7" max="7" width="8.69921875" customWidth="1"/>
+    <col min="8" max="8" width="16.296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -436,11 +439,11 @@
         <v>180300</v>
       </c>
       <c r="G2">
-        <v>1.974497499759309E-2</v>
+        <v>1.489130000845762E-2</v>
       </c>
       <c r="H2">
         <f>G2*1000</f>
-        <v>19.74497499759309</v>
+        <v>14.89130000845762</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -460,15 +463,15 @@
         <v>720600</v>
       </c>
       <c r="F3">
-        <f t="shared" ref="F3:F6" si="0">E3+D3+C3</f>
+        <f t="shared" ref="F3:F8" si="0">E3+D3+C3</f>
         <v>720600</v>
       </c>
       <c r="G3">
-        <v>7.6027349998184945E-2</v>
+        <v>6.4644099998986349E-2</v>
       </c>
       <c r="H3">
-        <f t="shared" ref="H3:H6" si="1">G3*1000</f>
-        <v>76.027349998184945</v>
+        <f t="shared" ref="H3:H8" si="1">G3*1000</f>
+        <v>64.644099998986349</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -492,11 +495,11 @@
         <v>2881200</v>
       </c>
       <c r="G4">
-        <v>0.2674020750055206</v>
+        <v>0.35485622500709718</v>
       </c>
       <c r="H4">
         <f t="shared" si="1"/>
-        <v>267.4020750055206</v>
+        <v>354.85622500709718</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -520,11 +523,11 @@
         <v>11522400</v>
       </c>
       <c r="G5">
-        <v>1.226032775004569</v>
+        <v>1.6166599999996829</v>
       </c>
       <c r="H5">
         <f t="shared" si="1"/>
-        <v>1226.032775004569</v>
+        <v>1616.6599999996829</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -548,11 +551,67 @@
         <v>46084800</v>
       </c>
       <c r="G6">
-        <v>7.0103948499963744</v>
+        <v>5.8685919499912416</v>
       </c>
       <c r="H6">
         <f t="shared" si="1"/>
-        <v>7010.3948499963744</v>
+        <v>5868.5919499912416</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>19200</v>
+      </c>
+      <c r="B7">
+        <v>19199</v>
+      </c>
+      <c r="C7">
+        <v>0</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+      <c r="E7">
+        <v>184329600</v>
+      </c>
+      <c r="F7">
+        <f t="shared" si="0"/>
+        <v>184329600</v>
+      </c>
+      <c r="G7">
+        <v>27.75740777501051</v>
+      </c>
+      <c r="H7">
+        <f t="shared" si="1"/>
+        <v>27757.40777501051</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>38400</v>
+      </c>
+      <c r="B8">
+        <v>38399</v>
+      </c>
+      <c r="C8">
+        <v>0</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+      <c r="E8">
+        <v>737299200</v>
+      </c>
+      <c r="F8">
+        <f t="shared" si="0"/>
+        <v>737299200</v>
+      </c>
+      <c r="G8">
+        <v>110.2417646250033</v>
+      </c>
+      <c r="H8">
+        <f t="shared" si="1"/>
+        <v>110241.7646250033</v>
       </c>
     </row>
   </sheetData>

</xml_diff>